<commit_message>
feat(parallel routes): use parallel links id as possible names
Signed-off-by: EstherLerouzic <esther.lerouzic@orange.com>
Change-Id: I9625573a16e203b2d75f0fcf2538332dd52f269f
</commit_message>
<xml_diff>
--- a/tests/data/parallel_omses/parallel_links.xlsx
+++ b/tests/data/parallel_omses/parallel_links.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\user\workspace\TIP\test\oopt-gnpy\tests\data\parallel_omses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA472786-6F8E-475D-B0E6-9CD49D2AF20B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED189B2C-35F9-4E9B-A822-7CA4A7630015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="20376" windowHeight="12096" tabRatio="500" activeTab="4" xr2:uid="{666FB473-79A7-47B9-AA02-762624321C5F}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="84">
   <si>
     <t>list of amps type_variety separated by ‘ | ’. amp type_variety must be defined in eqpt_config.json</t>
   </si>
@@ -319,10 +319,10 @@
     <t>std_medium_gain</t>
   </si>
   <si>
-    <t>Brest | Quimper</t>
-  </si>
-  <si>
-    <t>0 | 1</t>
+    <t>Lorient | Vannes</t>
+  </si>
+  <si>
+    <t>1 | 0</t>
   </si>
 </sst>
 </file>
@@ -1820,9 +1820,7 @@
       <c r="H6" s="22">
         <v>80</v>
       </c>
-      <c r="I6" s="21">
-        <v>1</v>
-      </c>
+      <c r="I6" s="29"/>
       <c r="J6" s="22" t="s">
         <v>82</v>
       </c>
@@ -1852,10 +1850,10 @@
       <c r="G7" s="22">
         <v>1</v>
       </c>
-      <c r="I7" s="21"/>
-      <c r="J7" s="21" t="s">
-        <v>82</v>
-      </c>
+      <c r="I7" s="21">
+        <v>0</v>
+      </c>
+      <c r="J7" s="30"/>
       <c r="L7" s="22">
         <v>200</v>
       </c>
@@ -1885,9 +1883,6 @@
       <c r="I8" s="29" t="s">
         <v>83</v>
       </c>
-      <c r="J8" s="29" t="s">
-        <v>82</v>
-      </c>
       <c r="L8" s="30">
         <v>200</v>
       </c>
@@ -1911,9 +1906,7 @@
       <c r="F9" s="22">
         <v>50</v>
       </c>
-      <c r="I9" s="21">
-        <v>1</v>
-      </c>
+      <c r="I9" s="21"/>
       <c r="L9" s="22">
         <v>60</v>
       </c>

</xml_diff>